<commit_message>
IP-Insolvenzakten: Hauptschuld und Sicherheiten lückenlos belegen (#612)
* feat(testakten): belege Hauptschuld und IP-Sicherheiten

* fix(testakten): halte Kreditbelege zeitlich konsistent

* fix(testakten): ergänze Download-Navigation
</commit_message>
<xml_diff>
--- a/testakten/filmrechte-sicherungsuebertragung-insolvenz-schwetzingen/01_Mandat/03_Chronologie.xlsx
+++ b/testakten/filmrechte-sicherungsuebertragung-insolvenz-schwetzingen/01_Mandat/03_Chronologie.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronologie" sheetId="1" r:id="Rcfb3ffe94e3d46e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Termine" sheetId="2" r:id="Rda310d50c5a84421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chronologie" sheetId="1" r:id="Ra8fbc1fe4b4648fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Termine" sheetId="2" r:id="Radcf829795344a60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -316,10 +316,10 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="33" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="45" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="33" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="37" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -434,188 +434,375 @@
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="14" t="str">
-        <x:v>07.05.2024</x:v>
+        <x:v>23.04.2024</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Drehbeginn Deidesheim</x:v>
+        <x:v>Ziehung PL-01 valutiert: 620.000 EUR</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>Produktionsteam</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>02_Produktion_Medien/02_Produktionsdossier.docx</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/10_Bankfreigabe_PL01_620000.pdf</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>Rohmaterialbestand</x:v>
+        <x:v>CP laut Checkliste erfüllt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="15" t="str">
-        <x:v>22.11.2024</x:v>
+        <x:v>07.05.2024</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>Rohschnitt abgenommen</x:v>
+        <x:v>Drehbeginn Deidesheim</x:v>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>Produzent / Regie</x:v>
+        <x:v>Produktionsteam</x:v>
       </x:c>
       <x:c r="D11" s="15" t="str">
-        <x:v>Schnittprotokoll</x:v>
+        <x:v>02_Produktion_Medien/02_Produktionsdossier.docx</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>keine Originaldatei in Akte</x:v>
+        <x:v>Rohmaterialbestand</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>21.02.2025</x:v>
+        <x:v>12.07.2024</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Sicherungsabtretung Forderungen</x:v>
+        <x:v>Ziehung PL-02 valutiert: 480.000 EUR</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
         <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>04_Finanzierung_Sicherheiten/04_Sicherungsabtretung_Lizenzforderungen.docx</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/12_Bankfreigabe_PL02_480000.pdf</x:v>
       </x:c>
       <x:c r="E12" s="14" t="str">
-        <x:v>Anzeige an alle Debitoren?</x:v>
+        <x:v>CP laut Checkliste erfüllt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="15" t="str">
-        <x:v>04.08.2025</x:v>
+        <x:v>22.11.2024</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
-        <x:v>Autorin beanstandet Verwertungsumfang</x:v>
+        <x:v>Rohschnitt abgenommen</x:v>
       </x:c>
       <x:c r="C13" s="15" t="str">
-        <x:v>Zobel / Produktion</x:v>
+        <x:v>Produzent / Regie</x:v>
       </x:c>
       <x:c r="D13" s="15" t="str">
-        <x:v>03_Rechtekette_Vertraege/09_Mail_Autorin_Rechteumfang.eml</x:v>
+        <x:v>Schnittprotokoll</x:v>
       </x:c>
       <x:c r="E13" s="15" t="str">
-        <x:v>Einordnung der Korrespondenz</x:v>
+        <x:v>keine Originaldatei in Akte</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>12.03.2026</x:v>
+        <x:v>29.11.2024</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>Festivalpremiere Heidelberg</x:v>
+        <x:v>Ziehung PL-03 valutiert: 420.000 EUR</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>Produktion / Publikum</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Presseunterlagen</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/14_Bankfreigabe_PL03_420000.pdf</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>verwendete Filmfassung</x:v>
+        <x:v>CP laut Checkliste erfüllt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="15" t="str">
-        <x:v>18.08.2026</x:v>
+        <x:v>10.01.2025</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>Zahlungsstockung angezeigt</x:v>
+        <x:v>Nachtrag Fertigstellungstranche 420.000 EUR</x:v>
       </x:c>
       <x:c r="C15" s="15" t="str">
-        <x:v>Produktion / Bank</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D15" s="15" t="str">
-        <x:v>Bankakte</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/08_Nachtrag_Fertigstellungstranche_2025.pdf</x:v>
       </x:c>
       <x:c r="E15" s="15" t="str">
-        <x:v>vollständige Liquiditätsdaten</x:v>
+        <x:v>zusätzliche Tranche</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>30.09.2026</x:v>
+        <x:v>15.01.2025</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Insolvenzverfahren eröffnet</x:v>
+        <x:v>Ziehung FT-01 valutiert: 250.000 EUR</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>AG Heidelberg / Dr. Berthold</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>06_Insolvenz_AssetDeal/01_Insolvenzeroeffnungsbeschluss.pdf</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/18_Bankfreigabe_FT01_250000.pdf</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>Rechtskraftvermerk</x:v>
+        <x:v>CP laut Checkliste erfüllt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="15" t="str">
-        <x:v>14.10.2026</x:v>
+        <x:v>21.02.2025</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>Bewertung Filmpaket</x:v>
+        <x:v>Sicherungsabtretung Forderungen</x:v>
       </x:c>
       <x:c r="C17" s="15" t="str">
-        <x:v>Neckarblick Valuation</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D17" s="15" t="str">
-        <x:v>06_Insolvenz_AssetDeal/03_Bewertung_Filmpaket.pdf</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/04_Sicherungsabtretung_Lizenzforderungen.docx</x:v>
       </x:c>
       <x:c r="E17" s="15" t="str">
-        <x:v>Rechteannahmen</x:v>
+        <x:v>Anzeige an alle Debitoren?</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
       <x:c r="A18" s="14" t="str">
-        <x:v>20.10.2026</x:v>
+        <x:v>04.04.2025</x:v>
       </x:c>
       <x:c r="B18" s="14" t="str">
-        <x:v>APA unterzeichnet</x:v>
+        <x:v>Ziehung PL-04 valutiert: 210.000 EUR</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Verwalterin / Weintor</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
-        <x:v>06_Insolvenz_AssetDeal/04_Asset_Purchase_Agreement_unterschrieben.docx</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/16_Bankfreigabe_PL04_210000.pdf</x:v>
       </x:c>
       <x:c r="E18" s="14" t="str">
-        <x:v>Verfügungs- und Zustimmungslage</x:v>
+        <x:v>Produktionslinie zu 1.730.000 EUR genutzt</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
       <x:c r="A19" s="15" t="str">
-        <x:v>21.10.2026</x:v>
+        <x:v>19.05.2025</x:v>
       </x:c>
       <x:c r="B19" s="15" t="str">
-        <x:v>Vollzug Bank angekündigt</x:v>
+        <x:v>Ziehung FT-02 valutiert: 170.000 EUR</x:v>
       </x:c>
       <x:c r="C19" s="15" t="str">
-        <x:v>Dr. Berthold / Palatina</x:v>
+        <x:v>Palatina / Kurpfalz Lichtbild</x:v>
       </x:c>
       <x:c r="D19" s="15" t="str">
-        <x:v>06_Insolvenz_AssetDeal/06_Mail_Verwalterin_Vollzugsankuendigung.eml</x:v>
+        <x:v>04_Finanzierung_Sicherheiten/20_Bankfreigabe_FT02_170000.pdf</x:v>
       </x:c>
       <x:c r="E19" s="15" t="str">
-        <x:v>Bankreaktion offen</x:v>
+        <x:v>Fertigstellungstranche voll genutzt</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="14" t="str">
+        <x:v>04.08.2025</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Autorin beanstandet Verwertungsumfang</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>Zobel / Produktion</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>03_Rechtekette_Vertraege/09_Mail_Autorin_Rechteumfang.eml</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="str">
+        <x:v>Einordnung der Korrespondenz</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="15" t="str">
+        <x:v>29.08.2025</x:v>
+      </x:c>
+      <x:c r="B21" s="15" t="str">
+        <x:v>Kapitalrückführung RZ-01: 180.000 EUR</x:v>
+      </x:c>
+      <x:c r="C21" s="15" t="str">
+        <x:v>Kurpfalz Lichtbild / Palatina</x:v>
+      </x:c>
+      <x:c r="D21" s="15" t="str">
+        <x:v>04_Finanzierung_Sicherheiten/21_Projektkontoauszug_Darlehen_und_Tilgungen.pdf</x:v>
+      </x:c>
+      <x:c r="E21" s="15" t="str">
+        <x:v>gebucht</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>15.02.2026</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>Kapitalrückführung RZ-02: 220.000 EUR</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>Kurpfalz Lichtbild / Palatina</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>04_Finanzierung_Sicherheiten/21_Projektkontoauszug_Darlehen_und_Tilgungen.pdf</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="str">
+        <x:v>gebucht</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="15" t="str">
+        <x:v>12.03.2026</x:v>
+      </x:c>
+      <x:c r="B23" s="15" t="str">
+        <x:v>Festivalpremiere Heidelberg</x:v>
+      </x:c>
+      <x:c r="C23" s="15" t="str">
+        <x:v>Produktion / Publikum</x:v>
+      </x:c>
+      <x:c r="D23" s="15" t="str">
+        <x:v>Presseunterlagen</x:v>
+      </x:c>
+      <x:c r="E23" s="15" t="str">
+        <x:v>verwendete Filmfassung</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>20.05.2026</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>Kapitalrückführung RZ-03: 310.000 EUR</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>Kurpfalz Lichtbild / Palatina</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>04_Finanzierung_Sicherheiten/21_Projektkontoauszug_Darlehen_und_Tilgungen.pdf</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>gebucht</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" customHeight="1">
+      <x:c r="A25" s="15" t="str">
+        <x:v>18.08.2026</x:v>
+      </x:c>
+      <x:c r="B25" s="15" t="str">
+        <x:v>Zahlungsstockung angezeigt</x:v>
+      </x:c>
+      <x:c r="C25" s="15" t="str">
+        <x:v>Produktion / Bank</x:v>
+      </x:c>
+      <x:c r="D25" s="15" t="str">
+        <x:v>Bankakte</x:v>
+      </x:c>
+      <x:c r="E25" s="15" t="str">
+        <x:v>vollständige Liquiditätsdaten</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="34" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>30.09.2026</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Insolvenzverfahren eröffnet</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>AG Heidelberg / Dr. Berthold</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>06_Insolvenz_AssetDeal/01_Insolvenzeroeffnungsbeschluss.pdf</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>Rechtskraftvermerk</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="34" customHeight="1">
+      <x:c r="A27" s="15" t="str">
+        <x:v>14.10.2026</x:v>
+      </x:c>
+      <x:c r="B27" s="15" t="str">
+        <x:v>Bewertung Filmpaket</x:v>
+      </x:c>
+      <x:c r="C27" s="15" t="str">
+        <x:v>Neckarblick Valuation</x:v>
+      </x:c>
+      <x:c r="D27" s="15" t="str">
+        <x:v>06_Insolvenz_AssetDeal/03_Bewertung_Filmpaket.pdf</x:v>
+      </x:c>
+      <x:c r="E27" s="15" t="str">
+        <x:v>Rechteannahmen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="34" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>20.10.2026</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>APA unterzeichnet</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>Verwalterin / Weintor</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>06_Insolvenz_AssetDeal/04_Asset_Purchase_Agreement_unterschrieben.docx</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>Verfügungs- und Zustimmungslage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="34" customHeight="1">
+      <x:c r="A29" s="15" t="str">
+        <x:v>21.10.2026</x:v>
+      </x:c>
+      <x:c r="B29" s="15" t="str">
+        <x:v>Vollzug Bank angekündigt</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>Dr. Berthold / Palatina</x:v>
+      </x:c>
+      <x:c r="D29" s="15" t="str">
+        <x:v>06_Insolvenz_AssetDeal/06_Mail_Verwalterin_Vollzugsankuendigung.eml</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str">
+        <x:v>Bankreaktion offen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="34" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>22.10.2026</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Saldo 1.476.830,44 EUR und Sicherungsfall angezeigt</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>Palatina / Dr. Berthold</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>04_Finanzierung_Sicherheiten/23_Aktueller_Saldennachweis_2026-10-22.pdf</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>Rechtswirkungen bleiben streitig</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" s="15" t="str">
         <x:v>29.10.2026</x:v>
       </x:c>
-      <x:c r="B20" s="14" t="str">
+      <x:c r="B31" s="15" t="str">
         <x:v>technische Übergabe geplant</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C31" s="15" t="str">
         <x:v>Verwalterin / Erwerberin</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="D31" s="15" t="str">
         <x:v>06_Insolvenz_AssetDeal/05_Closing_Checkliste.xlsx</x:v>
       </x:c>
-      <x:c r="E20" s="14" t="str">
+      <x:c r="E31" s="15" t="str">
         <x:v>Token, Master und Forderungslisten</x:v>
       </x:c>
     </x:row>

</xml_diff>